<commit_message>
Ajusta fluxo final e operador
</commit_message>
<xml_diff>
--- a/bot/data/respostas.xlsx
+++ b/bot/data/respostas.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerguntasRespostas" sheetId="1" r:id="R9a756608685f4b31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucoes" sheetId="2" r:id="Rd5f6915b50d646a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorias" sheetId="3" r:id="R173eca0f6e2243e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerguntasRespostas" sheetId="1" r:id="R5539f9586b4e4476"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucoes" sheetId="2" r:id="R59b48f1db9984961"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorias" sheetId="3" r:id="Rb49de8484c3d4c94"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -438,13 +438,7 @@
     <x:t xml:space="preserve">atendente</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Seu atendimento será encaminhado para um operador. Aguarde por favor.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">humano</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">humano;operador;suporte;pessoa;falar com atendente</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">reclamar</x:t>
@@ -612,13 +606,13 @@
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FFFFFF"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="14"/>
-      <x:color rgb="FFFFFF"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
@@ -636,17 +630,17 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="1F4E78"/>
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="D9EAF7"/>
+        <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="1F4E78"/>
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -2094,38 +2088,38 @@
       <x:c r="A48" s="2" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="B48" s="2" t="s">
+      <x:c r="B48" s="2" t="str">
+        <x:v>Aguarde um momento, um dos nossos operadores irá te atender.</x:v>
+      </x:c>
+      <x:c r="C48" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D48" s="2" t="s">
         <x:v>142</x:v>
-      </x:c>
-      <x:c r="C48" s="2" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="D48" s="2" t="s">
-        <x:v>143</x:v>
       </x:c>
       <x:c r="E48" s="2">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="F48" s="2" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="G48" s="2" t="s">
-        <x:v>144</x:v>
+      <x:c r="F48" s="2" t="str">
+        <x:v>sim</x:v>
+      </x:c>
+      <x:c r="G48" s="2" t="str">
+        <x:v>humano;operador;suporte;pessoa;falar com atendente;atendente;mano;falar com operador;falar com o operador;falar com alguem;quero falar com alguem;quero falar com operador;quero falar com o operador;quero falar com atendente;preciso falar com alguem;preciso falar com uma pessoa;chamar operador;chamar atendente</x:v>
       </x:c>
       <x:c r="H48" s="2"/>
     </x:row>
     <x:row r="49" ht="27.600000381469727">
       <x:c r="A49" s="2" t="s">
-        <x:v>145</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="B49" s="2" t="s">
-        <x:v>146</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="C49" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="D49" s="2" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="E49" s="2">
         <x:v>9</x:v>
@@ -2134,22 +2128,22 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="G49" s="2" t="s">
-        <x:v>147</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="H49" s="2"/>
     </x:row>
     <x:row r="50" ht="27.600000381469727">
       <x:c r="A50" s="2" t="s">
-        <x:v>148</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B50" s="2" t="s">
-        <x:v>149</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="C50" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="D50" s="2" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="E50" s="2">
         <x:v>8</x:v>
@@ -2158,22 +2152,22 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="G50" s="2" t="s">
-        <x:v>150</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="H50" s="2"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="2" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="B51" s="2" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="C51" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D51" s="2" t="s">
         <x:v>151</x:v>
-      </x:c>
-      <x:c r="B51" s="2" t="s">
-        <x:v>152</x:v>
-      </x:c>
-      <x:c r="C51" s="2" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="D51" s="2" t="s">
-        <x:v>153</x:v>
       </x:c>
       <x:c r="E51" s="2">
         <x:v>5</x:v>
@@ -2182,22 +2176,22 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G51" s="2" t="s">
-        <x:v>154</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="H51" s="2"/>
     </x:row>
     <x:row r="52" ht="27.600000381469727">
       <x:c r="A52" s="2" t="s">
-        <x:v>155</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="B52" s="2" t="s">
-        <x:v>156</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="C52" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
       <x:c r="D52" s="2" t="s">
-        <x:v>153</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="E52" s="2">
         <x:v>5</x:v>
@@ -2206,22 +2200,22 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G52" s="2" t="s">
-        <x:v>157</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="H52" s="2"/>
     </x:row>
     <x:row r="53" ht="41.400001525878906">
       <x:c r="A53" s="2" t="s">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="B53" s="2" t="s">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="C53" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D53" s="2" t="s">
         <x:v>158</x:v>
-      </x:c>
-      <x:c r="B53" s="2" t="s">
-        <x:v>159</x:v>
-      </x:c>
-      <x:c r="C53" s="2" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="D53" s="2" t="s">
-        <x:v>160</x:v>
       </x:c>
       <x:c r="E53" s="2">
         <x:v>1</x:v>
@@ -2230,7 +2224,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="G53" s="2" t="s">
-        <x:v>161</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="H53" s="2"/>
     </x:row>
@@ -2752,7 +2746,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f1236e0a4d140ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82c81b41cd8543dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2767,80 +2761,80 @@
   <x:sheetData>
     <x:row r="1" ht="22.350000381469727" customHeight="1">
       <x:c r="A1" s="5" t="s">
-        <x:v>162</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="B1" s="6"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="s">
-        <x:v>163</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="B2" t="s">
-        <x:v>164</x:v>
+        <x:v>162</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="s">
-        <x:v>165</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="B3" t="s">
-        <x:v>166</x:v>
+        <x:v>164</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="3" t="s">
-        <x:v>167</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B4" t="s">
-        <x:v>168</x:v>
+        <x:v>166</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="3" t="s">
-        <x:v>169</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B5" t="s">
-        <x:v>170</x:v>
+        <x:v>168</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="3" t="s">
-        <x:v>171</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="B6" t="s">
-        <x:v>172</x:v>
+        <x:v>170</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="3" t="s">
-        <x:v>173</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="B7" t="s">
-        <x:v>174</x:v>
+        <x:v>172</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="3" t="s">
-        <x:v>175</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="B8" t="s">
-        <x:v>176</x:v>
+        <x:v>174</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="3" t="s">
-        <x:v>177</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="B9" t="s">
-        <x:v>178</x:v>
+        <x:v>176</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="3" t="s">
-        <x:v>179</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B10" t="s">
-        <x:v>180</x:v>
+        <x:v>178</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2920,7 +2914,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B1" s="4" t="s">
-        <x:v>181</x:v>
+        <x:v>179</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -2928,7 +2922,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B2" t="s">
-        <x:v>182</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2936,7 +2930,7 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B3" t="s">
-        <x:v>183</x:v>
+        <x:v>181</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -2944,7 +2938,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B4" t="s">
-        <x:v>184</x:v>
+        <x:v>182</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -2952,7 +2946,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="B5" t="s">
-        <x:v>185</x:v>
+        <x:v>183</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2960,7 +2954,7 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="B6" t="s">
-        <x:v>186</x:v>
+        <x:v>184</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2968,7 +2962,7 @@
         <x:v>71</x:v>
       </x:c>
       <x:c r="B7" t="s">
-        <x:v>187</x:v>
+        <x:v>185</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2976,7 +2970,7 @@
         <x:v>89</x:v>
       </x:c>
       <x:c r="B8" t="s">
-        <x:v>188</x:v>
+        <x:v>186</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2984,7 +2978,7 @@
         <x:v>97</x:v>
       </x:c>
       <x:c r="B9" t="s">
-        <x:v>189</x:v>
+        <x:v>187</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2992,7 +2986,7 @@
         <x:v>111</x:v>
       </x:c>
       <x:c r="B10" t="s">
-        <x:v>190</x:v>
+        <x:v>188</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -3000,7 +2994,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="B11" t="s">
-        <x:v>191</x:v>
+        <x:v>189</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -3008,37 +3002,37 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B12" t="s">
-        <x:v>192</x:v>
+        <x:v>190</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B13" t="s">
-        <x:v>193</x:v>
+        <x:v>191</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="s">
-        <x:v>153</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B14" t="s">
-        <x:v>194</x:v>
+        <x:v>192</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="s">
-        <x:v>160</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B15" t="s">
-        <x:v>195</x:v>
+        <x:v>193</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa87abfe61c74f33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6979942085d45ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>